<commit_message>
Actualizar app, paso1, paso2, __init__, informes y listado jira
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/isoReport/docs/Informe_ISO_todas_solicitudes.xlsx
+++ b/isoReport/docs/Informe_ISO_todas_solicitudes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aagricola-my.sharepoint.com/personal/inavarro_atlanticaagricola_com/Documents/Escritorio/Repos/isoReport/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_A98EA00611652D80B024ADCFA9FBF10F0359CB53" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A027DD9-4115-4624-8BE3-AEA87714E290}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_A98EA00611652D80B024ADCFA9FBF10F0359CB53" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89297026-2C81-4F51-A217-5A651046961F}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="348" yWindow="3708" windowWidth="7080" windowHeight="4080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19000" yWindow="-10910" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
@@ -2926,7 +2926,8 @@
   <dimension ref="A1:D190"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.109375" customWidth="1"/>
+    <col min="1" max="1" width="39.5546875" customWidth="1"/>
+    <col min="2" max="2" width="255.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -10027,6 +10028,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="43.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
Actualizar app, editor, paso1; bbdd y solicitudes (solicitudes_2025.xlsx, bbdd_16.02.2026.json)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/isoReport/docs/Informe_ISO_todas_solicitudes.xlsx
+++ b/isoReport/docs/Informe_ISO_todas_solicitudes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aagricola-my.sharepoint.com/personal/inavarro_atlanticaagricola_com/Documents/Escritorio/Repos/isoReport/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="11_A98EA00611652D80B024ADCFA9FBF10F0359CB53" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89297026-2C81-4F51-A217-5A651046961F}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_A98EA00611652D80B024ADCFA9FBF10F0359CB53" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D90F5C9-8C31-4451-BD1C-AD3A020B3EF1}"/>
   <bookViews>
-    <workbookView xWindow="19000" yWindow="-10910" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
@@ -2926,7 +2926,7 @@
   <dimension ref="A1:D190"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.5546875" customWidth="1"/>
+    <col min="1" max="1" width="70.88671875" customWidth="1"/>
     <col min="2" max="2" width="255.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Actualizar app, editor, datos; bbdd 17.02.26, obsoleto, script rellenar_fecha_validacion_desde_jira
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/isoReport/docs/Informe_ISO_todas_solicitudes.xlsx
+++ b/isoReport/docs/Informe_ISO_todas_solicitudes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aagricola-my.sharepoint.com/personal/inavarro_atlanticaagricola_com/Documents/Escritorio/Repos/isoReport/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="11_A98EA00611652D80B024ADCFA9FBF10F0359CB53" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D90F5C9-8C31-4451-BD1C-AD3A020B3EF1}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_A98EA00611652D80B024ADCFA9FBF10F0359CB53" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E586C478-89CA-43D0-8821-10A018840525}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3622" uniqueCount="837">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3640" uniqueCount="838">
   <si>
     <t>Responsable:</t>
   </si>
@@ -2566,15 +2566,33 @@
   </si>
   <si>
     <t>7,5 - 8,5</t>
+  </si>
+  <si>
+    <t>Marketing y/o Dirección</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -2616,9 +2634,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2923,11 +2948,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D190"/>
+  <dimension ref="A1:D200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="70.88671875" customWidth="1"/>
-    <col min="2" max="2" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="54.77734375" customWidth="1"/>
+    <col min="3" max="3" width="70.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -4720,13 +4747,101 @@
         <v>145</v>
       </c>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A190" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B190" s="1"/>
+    <row r="190" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A190" s="2" t="s">
+        <v>815</v>
+      </c>
+      <c r="B190" s="2" t="s">
+        <v>826</v>
+      </c>
       <c r="C190" s="1"/>
       <c r="D190" s="1"/>
+    </row>
+    <row r="191" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A191" s="2" t="s">
+        <v>816</v>
+      </c>
+      <c r="B191" s="2" t="s">
+        <v>827</v>
+      </c>
+      <c r="C191" s="1"/>
+      <c r="D191" s="1"/>
+    </row>
+    <row r="192" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A192" s="2" t="s">
+        <v>817</v>
+      </c>
+      <c r="B192" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="C192" s="1"/>
+      <c r="D192" s="1"/>
+    </row>
+    <row r="193" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A193" s="2" t="s">
+        <v>818</v>
+      </c>
+      <c r="B193" s="2" t="s">
+        <v>829</v>
+      </c>
+      <c r="C193" s="1"/>
+      <c r="D193" s="1"/>
+    </row>
+    <row r="194" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A194" s="2" t="s">
+        <v>819</v>
+      </c>
+      <c r="B194" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="C194" s="1"/>
+      <c r="D194" s="1"/>
+    </row>
+    <row r="195" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A195" s="2" t="s">
+        <v>819</v>
+      </c>
+      <c r="B195" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="C195" s="1"/>
+      <c r="D195" s="1"/>
+    </row>
+    <row r="196" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A196" s="2" t="s">
+        <v>819</v>
+      </c>
+      <c r="B196" s="2" t="s">
+        <v>831</v>
+      </c>
+      <c r="C196" s="1"/>
+      <c r="D196" s="1"/>
+    </row>
+    <row r="197" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A197" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="B197" s="2" t="s">
+        <v>832</v>
+      </c>
+      <c r="C197" s="1"/>
+      <c r="D197" s="1"/>
+    </row>
+    <row r="198" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A198" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>833</v>
+      </c>
+      <c r="C198" s="1"/>
+      <c r="D198" s="1"/>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A200" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B200" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>